<commit_message>
ADD: split period logic
</commit_message>
<xml_diff>
--- a/SPLIT_COMPANY_DATA/RESULT/companies_result/OП ТАСРУД/OП ТАСРУД.xlsx
+++ b/SPLIT_COMPANY_DATA/RESULT/companies_result/OП ТАСРУД/OП ТАСРУД.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="29">
   <si>
     <t>Дата</t>
   </si>
@@ -53,9 +53,6 @@
   </si>
   <si>
     <t>Billing_Document</t>
-  </si>
-  <si>
-    <t>2026-05-13</t>
   </si>
   <si>
     <t>В2108СА</t>
@@ -110,8 +107,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -197,11 +195,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -209,9 +208,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -565,20 +564,20 @@
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" t="s">
-        <v>13</v>
+      <c r="A2" s="2">
+        <v>46155</v>
       </c>
       <c r="B2">
         <v>1146</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F2">
         <v>41.258</v>
@@ -596,7 +595,7 @@
         <v>73.44</v>
       </c>
       <c r="K2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -606,20 +605,20 @@
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" t="s">
-        <v>13</v>
+      <c r="A3" s="2">
+        <v>46155</v>
       </c>
       <c r="B3">
         <v>1148</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
         <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>18</v>
       </c>
       <c r="F3">
         <v>44.382</v>
@@ -637,7 +636,7 @@
         <v>79</v>
       </c>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -647,80 +646,80 @@
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="5">
+      <c r="A8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="6">
         <v>85.64</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="6">
         <v>2</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="6">
         <v>1.75</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="6">
         <v>149.87</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="6">
         <v>152.44</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="6">
         <v>2.57</v>
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="7">
+      <c r="A9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="8">
         <v>85.64</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="8">
         <v>2</v>
       </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7">
+      <c r="D9" s="8"/>
+      <c r="E9" s="8">
         <v>149.87</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="8">
         <v>152.44</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="8">
         <v>2.57</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ADD: note feature in the files
</commit_message>
<xml_diff>
--- a/SPLIT_COMPANY_DATA/RESULT/companies_result/OП ТАСРУД/OП ТАСРУД.xlsx
+++ b/SPLIT_COMPANY_DATA/RESULT/companies_result/OП ТАСРУД/OП ТАСРУД.xlsx
@@ -278,7 +278,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -288,12 +288,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9EAF7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFBDD7EE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -344,17 +338,17 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>

<commit_message>
ADD: new prices from 26.06.2026
</commit_message>
<xml_diff>
--- a/SPLIT_COMPANY_DATA/RESULT/companies_result/OП ТАСРУД/OП ТАСРУД.xlsx
+++ b/SPLIT_COMPANY_DATA/RESULT/companies_result/OП ТАСРУД/OП ТАСРУД.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="45">
   <si>
     <t>Дата</t>
   </si>
@@ -49,61 +49,88 @@
     <t>Час</t>
   </si>
   <si>
-    <t>Километри</t>
-  </si>
-  <si>
-    <t>Billing_Document</t>
-  </si>
-  <si>
-    <t>Варна Порт</t>
-  </si>
-  <si>
     <t>Варна Варненчик</t>
   </si>
   <si>
-    <t>Варна Цар Освободител</t>
+    <t>Варна Чайка</t>
+  </si>
+  <si>
+    <t>Варна</t>
+  </si>
+  <si>
+    <t>Варна Сливница</t>
+  </si>
+  <si>
+    <t>В9846КН</t>
+  </si>
+  <si>
+    <t>ТУБА ТАСРУД2</t>
   </si>
   <si>
     <t>В2075СА</t>
   </si>
   <si>
+    <t>В7853КР</t>
+  </si>
+  <si>
+    <t>В3528НН</t>
+  </si>
+  <si>
+    <t>В7232ВР</t>
+  </si>
+  <si>
     <t>В2108СА</t>
   </si>
   <si>
-    <t>ТУБАТАСРУД1</t>
-  </si>
-  <si>
-    <t>В1485РР</t>
+    <t>78970155027720592</t>
+  </si>
+  <si>
+    <t>78970155027720683</t>
   </si>
   <si>
     <t>78970155027720626</t>
   </si>
   <si>
+    <t>78970155027720600</t>
+  </si>
+  <si>
+    <t>78970155027720667</t>
+  </si>
+  <si>
+    <t>78970155027720634</t>
+  </si>
+  <si>
     <t>78970155027720642</t>
   </si>
   <si>
-    <t>78970155027720675</t>
-  </si>
-  <si>
-    <t>78970155027720618</t>
-  </si>
-  <si>
     <t>DIESEL EKONOMY</t>
   </si>
   <si>
     <t>95 EKONOMY UNLEADED</t>
   </si>
   <si>
-    <t>15:40</t>
-  </si>
-  <si>
-    <t>15:26</t>
-  </si>
-  <si>
-    <t>15:09</t>
-  </si>
-  <si>
-    <t>15:10</t>
+    <t>E GAS LPG</t>
+  </si>
+  <si>
+    <t>2026-06-17 09:05:16</t>
+  </si>
+  <si>
+    <t>2026-06-17 09:05:29</t>
+  </si>
+  <si>
+    <t>2026-06-17 09:27:04</t>
+  </si>
+  <si>
+    <t>2026-06-18 14:18:12</t>
+  </si>
+  <si>
+    <t>2026-06-23 10:46:50</t>
+  </si>
+  <si>
+    <t>2026-06-24 13:58:54</t>
+  </si>
+  <si>
+    <t>2026-06-25 15:29:07</t>
   </si>
   <si>
     <t>Общи литри по продукт / OП ТАСРУД</t>
@@ -523,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -536,12 +563,10 @@
     <col min="8" max="8" width="23.7109375" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="23.7109375" customWidth="1"/>
-    <col min="11" max="11" width="7.7109375" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" customWidth="1"/>
+    <col min="11" max="11" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:11">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -575,268 +600,363 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="3">
+        <v>46190</v>
+      </c>
+      <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2">
+        <v>36.15</v>
+      </c>
+      <c r="G2" s="1">
+        <v>1.56</v>
+      </c>
+      <c r="H2">
+        <v>56.39</v>
+      </c>
+      <c r="I2" s="1">
+        <v>1.59</v>
+      </c>
+      <c r="J2">
+        <v>57.48</v>
+      </c>
+      <c r="K2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="3">
+        <v>46190</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3">
+        <v>3.49</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1.52</v>
+      </c>
+      <c r="H3">
+        <v>5.3</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1.55</v>
+      </c>
+      <c r="J3">
+        <v>5.41</v>
+      </c>
+      <c r="K3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="3">
+        <v>46190</v>
+      </c>
+      <c r="B4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="3">
-        <v>46180</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4">
+        <v>50</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1.56</v>
+      </c>
+      <c r="H4">
+        <v>78</v>
+      </c>
+      <c r="I4" s="1">
+        <v>1.59</v>
+      </c>
+      <c r="J4">
+        <v>79.5</v>
+      </c>
+      <c r="K4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="3">
+        <v>46191</v>
+      </c>
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5">
+        <v>44.69</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1.52</v>
+      </c>
+      <c r="H5">
+        <v>67.93000000000001</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1.55</v>
+      </c>
+      <c r="J5">
+        <v>69.27</v>
+      </c>
+      <c r="K5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="3">
+        <v>46196</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6">
+        <v>63.95</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1.49</v>
+      </c>
+      <c r="H6">
+        <v>95.29000000000001</v>
+      </c>
+      <c r="I6" s="1">
+        <v>1.52</v>
+      </c>
+      <c r="J6">
+        <v>97.2</v>
+      </c>
+      <c r="K6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="3">
+        <v>46197</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="E2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2">
-        <v>45.66</v>
-      </c>
-      <c r="G2" s="1">
-        <v>1.61</v>
-      </c>
-      <c r="H2">
-        <v>73.51000000000001</v>
-      </c>
-      <c r="I2" s="1">
-        <v>1.64</v>
-      </c>
-      <c r="J2">
-        <v>74.88</v>
-      </c>
-      <c r="K2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>216026</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="3">
-        <v>46182</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7">
+        <v>26.58</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="H7">
+        <v>17.28</v>
+      </c>
+      <c r="I7" s="1">
+        <v>0.66</v>
+      </c>
+      <c r="J7">
+        <v>17.54</v>
+      </c>
+      <c r="K7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="3">
+        <v>46198</v>
+      </c>
+      <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C8" t="s">
         <v>21</v>
       </c>
-      <c r="E3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3">
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8">
+        <v>43.92</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1.48</v>
+      </c>
+      <c r="H8">
+        <v>65</v>
+      </c>
+      <c r="I8" s="1">
+        <v>1.51</v>
+      </c>
+      <c r="J8">
+        <v>66.31999999999999</v>
+      </c>
+      <c r="K8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G3" s="1">
-        <v>1.61</v>
-      </c>
-      <c r="H3">
-        <v>64.40000000000001</v>
-      </c>
-      <c r="I3" s="1">
-        <v>1.64</v>
-      </c>
-      <c r="J3">
-        <v>65.59999999999999</v>
-      </c>
-      <c r="K3" t="s">
-        <v>27</v>
-      </c>
-      <c r="L3">
-        <v>80850</v>
-      </c>
-      <c r="M3">
-        <v>196031</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="3">
-        <v>46185</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4">
-        <v>10.02</v>
-      </c>
-      <c r="G4" s="1">
-        <v>1.53</v>
-      </c>
-      <c r="H4">
-        <v>15.33</v>
-      </c>
-      <c r="I4" s="1">
-        <v>1.56</v>
-      </c>
-      <c r="J4">
-        <v>15.63</v>
-      </c>
-      <c r="K4" t="s">
-        <v>28</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>274702</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="3">
-        <v>46185</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5">
-        <v>54.88</v>
-      </c>
-      <c r="G5" s="1">
-        <v>1.58</v>
-      </c>
-      <c r="H5">
-        <v>86.70999999999999</v>
-      </c>
-      <c r="I5" s="1">
-        <v>1.61</v>
-      </c>
-      <c r="J5">
-        <v>88.36</v>
-      </c>
-      <c r="K5" t="s">
+      <c r="B12" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>274704</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="A8" s="4" t="s">
+      <c r="B13" s="7">
+        <v>194.02</v>
+      </c>
+      <c r="C13" s="7">
+        <v>4</v>
+      </c>
+      <c r="D13" s="8">
+        <v>1.5188</v>
+      </c>
+      <c r="E13" s="7">
+        <v>294.68</v>
+      </c>
+      <c r="F13" s="7">
+        <v>300.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-    </row>
-    <row r="9" spans="1:13">
-      <c r="A9" s="5" t="s">
+      <c r="B14" s="7">
+        <v>48.18</v>
+      </c>
+      <c r="C14" s="7">
+        <v>2</v>
+      </c>
+      <c r="D14" s="8">
+        <v>1.5199</v>
+      </c>
+      <c r="E14" s="7">
+        <v>73.23</v>
+      </c>
+      <c r="F14" s="7">
+        <v>74.68000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" s="5" t="s">
+      <c r="B15" s="7">
+        <v>26.58</v>
+      </c>
+      <c r="C15" s="7">
+        <v>1</v>
+      </c>
+      <c r="D15" s="8">
+        <v>0.6501</v>
+      </c>
+      <c r="E15" s="7">
+        <v>17.28</v>
+      </c>
+      <c r="F15" s="7">
+        <v>17.54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="10">
+        <v>268.78</v>
+      </c>
+      <c r="C16" s="10">
         <v>7</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="7">
-        <v>140.54</v>
-      </c>
-      <c r="C10" s="7">
-        <v>3</v>
-      </c>
-      <c r="D10" s="8">
-        <v>1.5983</v>
-      </c>
-      <c r="E10" s="7">
-        <v>224.62</v>
-      </c>
-      <c r="F10" s="7">
-        <v>228.84</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
-      <c r="A11" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="7">
-        <v>10.02</v>
-      </c>
-      <c r="C11" s="7">
-        <v>1</v>
-      </c>
-      <c r="D11" s="8">
-        <v>1.5299</v>
-      </c>
-      <c r="E11" s="7">
-        <v>15.33</v>
-      </c>
-      <c r="F11" s="7">
-        <v>15.63</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
-      <c r="A12" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="10">
-        <v>150.56</v>
-      </c>
-      <c r="C12" s="10">
-        <v>4</v>
-      </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="10">
-        <v>239.95</v>
-      </c>
-      <c r="F12" s="10">
-        <v>244.47</v>
+      <c r="D16" s="8"/>
+      <c r="E16" s="10">
+        <v>385.19</v>
+      </c>
+      <c r="F16" s="10">
+        <v>392.72</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A11:F11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
ADD: new prices from 08072026
</commit_message>
<xml_diff>
--- a/SPLIT_COMPANY_DATA/RESULT/companies_result/OП ТАСРУД/OП ТАСРУД.xlsx
+++ b/SPLIT_COMPANY_DATA/RESULT/companies_result/OП ТАСРУД/OП ТАСРУД.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="55">
   <si>
     <t>Дата</t>
   </si>
@@ -34,9 +34,6 @@
     <t>Литри</t>
   </si>
   <si>
-    <t>Тип количество</t>
-  </si>
-  <si>
     <t>GTA цена</t>
   </si>
   <si>
@@ -58,19 +55,19 @@
     <t>Billing_Document</t>
   </si>
   <si>
-    <t>1147 Варна Ситроен</t>
-  </si>
-  <si>
-    <t>1158 Варна Чайка</t>
-  </si>
-  <si>
-    <t>1199 Varna Car Osvoboditel</t>
-  </si>
-  <si>
-    <t>1146 Варна Сливница</t>
-  </si>
-  <si>
-    <t>1148 Варна пристанище</t>
+    <t>Варна Варненчик</t>
+  </si>
+  <si>
+    <t>Варна Чайка</t>
+  </si>
+  <si>
+    <t>Варна Порт</t>
+  </si>
+  <si>
+    <t>Варна</t>
+  </si>
+  <si>
+    <t>Варна Сливница</t>
   </si>
   <si>
     <t>В9846КН</t>
@@ -130,82 +127,40 @@
     <t>E GAS LPG</t>
   </si>
   <si>
-    <t>L15</t>
-  </si>
-  <si>
-    <t>09:05:00</t>
-  </si>
-  <si>
-    <t>09:27:00</t>
-  </si>
-  <si>
-    <t>14:17:00</t>
-  </si>
-  <si>
-    <t>10:47:00</t>
-  </si>
-  <si>
-    <t>13:58:00</t>
-  </si>
-  <si>
-    <t>15:29:00</t>
-  </si>
-  <si>
-    <t>14:15:00</t>
-  </si>
-  <si>
-    <t>11:58:00</t>
-  </si>
-  <si>
-    <t>13:31:00</t>
-  </si>
-  <si>
-    <t>11:23:00</t>
-  </si>
-  <si>
-    <t>09:32:00</t>
-  </si>
-  <si>
-    <t>13:13:00</t>
-  </si>
-  <si>
-    <t>3233470868 3233470868</t>
-  </si>
-  <si>
-    <t>3233475738 3233475738</t>
-  </si>
-  <si>
-    <t>3233471450 3233471450</t>
-  </si>
-  <si>
-    <t>3233540873 3233540873</t>
-  </si>
-  <si>
-    <t>3233773957 3233773957</t>
-  </si>
-  <si>
-    <t>3233796170 3233796170</t>
-  </si>
-  <si>
-    <t>3233833855 3233833855</t>
-  </si>
-  <si>
-    <t>3233902234 3233902234</t>
-  </si>
-  <si>
-    <t>3234037747 3234037747</t>
-  </si>
-  <si>
-    <t>3234055345 3234055345</t>
-  </si>
-  <si>
-    <t>3234066509 3234066509</t>
-  </si>
-  <si>
-    <t>3234082075 3234082075</t>
-  </si>
-  <si>
-    <t>3234106919 3234106919</t>
+    <t>09:05</t>
+  </si>
+  <si>
+    <t>09:27</t>
+  </si>
+  <si>
+    <t>14:19</t>
+  </si>
+  <si>
+    <t>10:47</t>
+  </si>
+  <si>
+    <t>13:58</t>
+  </si>
+  <si>
+    <t>15:29</t>
+  </si>
+  <si>
+    <t>14:15</t>
+  </si>
+  <si>
+    <t>11:23</t>
+  </si>
+  <si>
+    <t>11:57</t>
+  </si>
+  <si>
+    <t>13:32</t>
+  </si>
+  <si>
+    <t>09:32</t>
+  </si>
+  <si>
+    <t>13:13</t>
   </si>
   <si>
     <t>Общи литри по продукт / OП ТАСРУД</t>
@@ -625,7 +580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -634,17 +589,16 @@
     <col min="4" max="4" width="28.7109375" customWidth="1"/>
     <col min="5" max="5" width="22.7109375" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="23.7109375" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="23.7109375" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" customWidth="1"/>
-    <col min="14" max="14" width="23.7109375" customWidth="1"/>
+    <col min="11" max="11" width="7.7109375" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:13">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -684,187 +638,172 @@
       <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="3">
         <v>46190</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F2">
         <v>36.15</v>
       </c>
-      <c r="G2" t="s">
-        <v>38</v>
+      <c r="G2" s="1">
+        <v>1.56</v>
       </c>
       <c r="H2">
-        <v>1.56</v>
+        <v>56.39</v>
       </c>
       <c r="I2" s="1">
-        <v>56.39</v>
+        <v>1.59</v>
       </c>
       <c r="J2">
-        <v>1.59</v>
-      </c>
-      <c r="K2" s="1">
         <v>57.48</v>
       </c>
-      <c r="L2" t="s">
-        <v>39</v>
+      <c r="K2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>115795</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="3">
         <v>46190</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F3">
         <v>3.49</v>
       </c>
-      <c r="G3" t="s">
-        <v>38</v>
+      <c r="G3" s="1">
+        <v>1.52</v>
       </c>
       <c r="H3">
-        <v>1.52</v>
+        <v>5.3</v>
       </c>
       <c r="I3" s="1">
-        <v>5.3</v>
+        <v>1.55</v>
       </c>
       <c r="J3">
-        <v>1.55</v>
-      </c>
-      <c r="K3" s="1">
         <v>5.41</v>
       </c>
-      <c r="L3" t="s">
-        <v>39</v>
+      <c r="K3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
       </c>
       <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
+        <v>115796</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="3">
         <v>46190</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F4">
         <v>50</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="1">
+        <v>1.56</v>
+      </c>
+      <c r="H4">
+        <v>78</v>
+      </c>
+      <c r="I4" s="1">
+        <v>1.59</v>
+      </c>
+      <c r="J4">
+        <v>79.5</v>
+      </c>
+      <c r="K4" t="s">
         <v>38</v>
       </c>
-      <c r="H4">
-        <v>1.56</v>
-      </c>
-      <c r="I4" s="1">
-        <v>78</v>
-      </c>
-      <c r="J4">
-        <v>1.59</v>
-      </c>
-      <c r="K4" s="1">
-        <v>79.5</v>
-      </c>
-      <c r="L4" t="s">
-        <v>40</v>
+      <c r="L4">
+        <v>8641</v>
       </c>
       <c r="M4">
-        <v>8641</v>
-      </c>
-      <c r="N4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
+        <v>114302</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="3">
         <v>46191</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F5">
         <v>44.69</v>
       </c>
-      <c r="G5" t="s">
-        <v>38</v>
+      <c r="G5" s="1">
+        <v>1.52</v>
       </c>
       <c r="H5">
-        <v>1.52</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="I5" s="1">
-        <v>67.93000000000001</v>
+        <v>1.55</v>
       </c>
       <c r="J5">
-        <v>1.55</v>
-      </c>
-      <c r="K5" s="1">
         <v>69.27</v>
       </c>
-      <c r="L5" t="s">
-        <v>41</v>
+      <c r="K5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L5">
+        <v>57750</v>
       </c>
       <c r="M5">
-        <v>173704</v>
-      </c>
-      <c r="N5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
+        <v>276331</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="3">
         <v>46196</v>
       </c>
@@ -872,43 +811,40 @@
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F6">
         <v>63.95</v>
       </c>
-      <c r="G6" t="s">
-        <v>38</v>
+      <c r="G6" s="1">
+        <v>1.49</v>
       </c>
       <c r="H6">
-        <v>1.49</v>
+        <v>95.29000000000001</v>
       </c>
       <c r="I6" s="1">
-        <v>95.29000000000001</v>
+        <v>1.52</v>
       </c>
       <c r="J6">
-        <v>1.52</v>
-      </c>
-      <c r="K6" s="1">
         <v>97.2</v>
       </c>
-      <c r="L6" t="s">
-        <v>42</v>
+      <c r="K6" t="s">
+        <v>40</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
       </c>
       <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
+        <v>277642</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" s="3">
         <v>46197</v>
       </c>
@@ -916,43 +852,40 @@
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F7">
         <v>26.58</v>
       </c>
-      <c r="G7" t="s">
-        <v>38</v>
+      <c r="G7" s="1">
+        <v>0.65</v>
       </c>
       <c r="H7">
-        <v>0.65</v>
+        <v>17.28</v>
       </c>
       <c r="I7" s="1">
-        <v>17.28</v>
+        <v>0.66</v>
       </c>
       <c r="J7">
-        <v>0.66</v>
-      </c>
-      <c r="K7" s="1">
         <v>17.54</v>
       </c>
-      <c r="L7" t="s">
-        <v>43</v>
+      <c r="K7" t="s">
+        <v>41</v>
+      </c>
+      <c r="L7">
+        <v>72290</v>
       </c>
       <c r="M7">
-        <v>72290</v>
-      </c>
-      <c r="N7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
+        <v>145223</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" s="3">
         <v>46198</v>
       </c>
@@ -960,43 +893,40 @@
         <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F8">
         <v>43.92</v>
       </c>
-      <c r="G8" t="s">
-        <v>38</v>
+      <c r="G8" s="1">
+        <v>1.48</v>
       </c>
       <c r="H8">
-        <v>1.48</v>
+        <v>65</v>
       </c>
       <c r="I8" s="1">
-        <v>65</v>
+        <v>1.51</v>
       </c>
       <c r="J8">
-        <v>1.51</v>
-      </c>
-      <c r="K8" s="1">
         <v>66.31999999999999</v>
       </c>
-      <c r="L8" t="s">
-        <v>44</v>
+      <c r="K8" t="s">
+        <v>42</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
       </c>
       <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
+        <v>145685</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" s="3">
         <v>46199</v>
       </c>
@@ -1004,219 +934,204 @@
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F9">
         <v>36.26</v>
       </c>
-      <c r="G9" t="s">
-        <v>38</v>
+      <c r="G9" s="1">
+        <v>1.48</v>
       </c>
       <c r="H9">
-        <v>1.48</v>
+        <v>53.66</v>
       </c>
       <c r="I9" s="1">
-        <v>53.66</v>
+        <v>1.51</v>
       </c>
       <c r="J9">
-        <v>1.51</v>
-      </c>
-      <c r="K9" s="1">
         <v>54.75</v>
       </c>
-      <c r="L9" t="s">
-        <v>45</v>
+      <c r="K9" t="s">
+        <v>43</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
       </c>
       <c r="M9">
-        <v>0</v>
-      </c>
-      <c r="N9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
+        <v>146073</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" s="3">
         <v>46202</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F10">
-        <v>20.45</v>
-      </c>
-      <c r="G10" t="s">
-        <v>38</v>
+        <v>9.83</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1.47</v>
       </c>
       <c r="H10">
-        <v>1.47</v>
+        <v>14.45</v>
       </c>
       <c r="I10" s="1">
-        <v>30.06</v>
+        <v>1.5</v>
       </c>
       <c r="J10">
-        <v>1.5</v>
-      </c>
-      <c r="K10" s="1">
-        <v>30.67</v>
-      </c>
-      <c r="L10" t="s">
-        <v>46</v>
+        <v>14.74</v>
+      </c>
+      <c r="K10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
       </c>
       <c r="M10">
-        <v>173856</v>
-      </c>
-      <c r="N10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
+        <v>279276</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" s="3">
         <v>46202</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F11">
-        <v>3.56</v>
-      </c>
-      <c r="G11" t="s">
-        <v>38</v>
+        <v>20.45</v>
+      </c>
+      <c r="G11" s="1">
+        <v>1.47</v>
       </c>
       <c r="H11">
-        <v>1.47</v>
+        <v>30.06</v>
       </c>
       <c r="I11" s="1">
-        <v>5.23</v>
+        <v>1.5</v>
       </c>
       <c r="J11">
-        <v>1.5</v>
-      </c>
-      <c r="K11" s="1">
-        <v>5.34</v>
-      </c>
-      <c r="L11" t="s">
-        <v>47</v>
+        <v>30.67</v>
+      </c>
+      <c r="K11" t="s">
+        <v>45</v>
+      </c>
+      <c r="L11">
+        <v>173856</v>
       </c>
       <c r="M11">
-        <v>49740</v>
-      </c>
-      <c r="N11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
+        <v>146416</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" s="3">
         <v>46202</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F12">
-        <v>17.47</v>
-      </c>
-      <c r="G12" t="s">
-        <v>38</v>
+        <v>3.56</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1.47</v>
       </c>
       <c r="H12">
-        <v>0.65</v>
+        <v>5.23</v>
       </c>
       <c r="I12" s="1">
-        <v>11.36</v>
+        <v>1.5</v>
       </c>
       <c r="J12">
-        <v>0.66</v>
-      </c>
-      <c r="K12" s="1">
-        <v>11.53</v>
-      </c>
-      <c r="L12" t="s">
-        <v>47</v>
+        <v>5.34</v>
+      </c>
+      <c r="K12" t="s">
+        <v>46</v>
+      </c>
+      <c r="L12">
+        <v>49740</v>
       </c>
       <c r="M12">
-        <v>49740</v>
-      </c>
-      <c r="N12" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
+        <v>121040</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13" s="3">
         <v>46202</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E13" t="s">
         <v>36</v>
       </c>
       <c r="F13">
-        <v>9.83</v>
-      </c>
-      <c r="G13" t="s">
-        <v>38</v>
+        <v>17.47</v>
+      </c>
+      <c r="G13" s="1">
+        <v>0.65</v>
       </c>
       <c r="H13">
-        <v>1.47</v>
+        <v>11.36</v>
       </c>
       <c r="I13" s="1">
-        <v>14.45</v>
+        <v>0.66</v>
       </c>
       <c r="J13">
-        <v>1.5</v>
-      </c>
-      <c r="K13" s="1">
-        <v>14.74</v>
-      </c>
-      <c r="L13" t="s">
-        <v>48</v>
+        <v>11.53</v>
+      </c>
+      <c r="K13" t="s">
+        <v>46</v>
+      </c>
+      <c r="L13">
+        <v>90526</v>
       </c>
       <c r="M13">
-        <v>0</v>
-      </c>
-      <c r="N13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
+        <v>121040</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
       <c r="A14" s="3">
         <v>46203</v>
       </c>
@@ -1224,89 +1139,83 @@
         <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F14">
         <v>46.26</v>
       </c>
-      <c r="G14" t="s">
-        <v>38</v>
+      <c r="G14" s="1">
+        <v>1.48</v>
       </c>
       <c r="H14">
-        <v>1.48</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="I14" s="1">
-        <v>68.45999999999999</v>
+        <v>1.51</v>
       </c>
       <c r="J14">
-        <v>1.51</v>
-      </c>
-      <c r="K14" s="1">
         <v>69.84999999999999</v>
       </c>
-      <c r="L14" t="s">
-        <v>49</v>
+      <c r="K14" t="s">
+        <v>47</v>
+      </c>
+      <c r="L14">
+        <v>86955</v>
       </c>
       <c r="M14">
-        <v>86955</v>
-      </c>
-      <c r="N14" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
+        <v>146737</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15" s="3">
         <v>46203</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F15">
         <v>18</v>
       </c>
-      <c r="G15" t="s">
-        <v>38</v>
+      <c r="G15" s="1">
+        <v>1.48</v>
       </c>
       <c r="H15">
-        <v>1.48</v>
+        <v>26.64</v>
       </c>
       <c r="I15" s="1">
-        <v>26.64</v>
+        <v>1.51</v>
       </c>
       <c r="J15">
-        <v>1.51</v>
-      </c>
-      <c r="K15" s="1">
         <v>27.18</v>
       </c>
-      <c r="L15" t="s">
-        <v>50</v>
+      <c r="K15" t="s">
+        <v>48</v>
+      </c>
+      <c r="L15">
+        <v>81420</v>
       </c>
       <c r="M15">
-        <v>81420</v>
-      </c>
-      <c r="N15" t="s">
-        <v>63</v>
+        <v>226009</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="4" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -1316,27 +1225,27 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="5" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20" s="7">
         <v>294.54</v>
@@ -1356,7 +1265,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B21" s="7">
         <v>82.02</v>
@@ -1376,7 +1285,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B22" s="7">
         <v>44.05</v>
@@ -1396,7 +1305,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="9" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B23" s="10">
         <v>420.61</v>

</xml_diff>

<commit_message>
ADD: new excel sheet for data analysis
</commit_message>
<xml_diff>
--- a/SPLIT_COMPANY_DATA/RESULT/companies_result/OП ТАСРУД/OП ТАСРУД.xlsx
+++ b/SPLIT_COMPANY_DATA/RESULT/companies_result/OП ТАСРУД/OП ТАСРУД.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="79">
   <si>
     <t>Дата</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>Тип количество</t>
+  </si>
+  <si>
+    <t>Базова ЕКО цена</t>
   </si>
   <si>
     <t>GTA цена</t>
@@ -649,7 +652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -662,13 +665,13 @@
     <col min="8" max="8" width="23.7109375" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="23.7109375" customWidth="1"/>
-    <col min="11" max="11" width="15.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" customWidth="1"/>
-    <col min="14" max="14" width="23.7109375" customWidth="1"/>
+    <col min="11" max="12" width="15.7109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" customWidth="1"/>
+    <col min="14" max="14" width="11.7109375" customWidth="1"/>
+    <col min="15" max="15" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -711,714 +714,765 @@
       <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" s="3">
         <v>46221</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2">
         <v>49</v>
       </c>
       <c r="G2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H2">
+        <v>1.528</v>
+      </c>
+      <c r="I2" s="1">
         <v>1.62</v>
       </c>
-      <c r="I2" s="1">
+      <c r="J2">
         <v>79.38</v>
       </c>
-      <c r="J2">
+      <c r="K2" s="1">
         <v>1.65</v>
       </c>
-      <c r="K2" s="1">
+      <c r="L2" s="1">
         <v>80.84999999999999</v>
       </c>
-      <c r="L2" t="s">
-        <v>40</v>
-      </c>
-      <c r="M2">
+      <c r="M2" t="s">
+        <v>41</v>
+      </c>
+      <c r="N2">
         <v>87457</v>
       </c>
-      <c r="N2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+      <c r="O2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" s="3">
         <v>46223</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F3">
-        <v>29.06</v>
+        <v>29.063</v>
       </c>
       <c r="G3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1">
         <v>0.63</v>
       </c>
-      <c r="I3" s="1">
-        <v>18.31</v>
-      </c>
       <c r="J3">
+        <v>18.30969</v>
+      </c>
+      <c r="K3" s="1">
         <v>0.64</v>
       </c>
-      <c r="K3" s="1">
-        <v>18.6</v>
-      </c>
-      <c r="L3" t="s">
-        <v>41</v>
-      </c>
-      <c r="M3">
+      <c r="L3" s="1">
+        <v>18.60032</v>
+      </c>
+      <c r="M3" t="s">
+        <v>42</v>
+      </c>
+      <c r="N3">
         <v>49934</v>
       </c>
-      <c r="N3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
+      <c r="O3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" s="3">
         <v>46223</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F4">
         <v>39</v>
       </c>
       <c r="G4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H4">
+        <v>1.546</v>
+      </c>
+      <c r="I4" s="1">
         <v>1.65</v>
       </c>
-      <c r="I4" s="1">
+      <c r="J4">
         <v>64.34999999999999</v>
       </c>
-      <c r="J4">
+      <c r="K4" s="1">
         <v>1.68</v>
       </c>
-      <c r="K4" s="1">
+      <c r="L4" s="1">
         <v>65.52</v>
       </c>
-      <c r="L4" t="s">
-        <v>42</v>
-      </c>
-      <c r="M4">
+      <c r="M4" t="s">
+        <v>43</v>
+      </c>
+      <c r="N4">
         <v>82093</v>
       </c>
-      <c r="N4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
+      <c r="O4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" s="3">
         <v>46224</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F5">
         <v>3.83</v>
       </c>
       <c r="G5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H5">
+        <v>1.389</v>
+      </c>
+      <c r="I5" s="1">
         <v>1.5</v>
       </c>
-      <c r="I5" s="1">
-        <v>5.74</v>
-      </c>
       <c r="J5">
+        <v>5.745</v>
+      </c>
+      <c r="K5" s="1">
         <v>1.53</v>
       </c>
-      <c r="K5" s="1">
-        <v>5.86</v>
-      </c>
-      <c r="L5" t="s">
-        <v>43</v>
-      </c>
-      <c r="M5">
+      <c r="L5" s="1">
+        <v>5.8599</v>
+      </c>
+      <c r="M5" t="s">
+        <v>44</v>
+      </c>
+      <c r="N5">
         <v>0</v>
       </c>
-      <c r="N5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14">
+      <c r="O5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" s="3">
         <v>46224</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F6">
         <v>20</v>
       </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H6">
+        <v>1.564</v>
+      </c>
+      <c r="I6" s="1">
         <v>1.65</v>
       </c>
-      <c r="I6" s="1">
+      <c r="J6">
         <v>33</v>
       </c>
-      <c r="J6">
+      <c r="K6" s="1">
         <v>1.68</v>
       </c>
-      <c r="K6" s="1">
+      <c r="L6" s="1">
         <v>33.6</v>
       </c>
-      <c r="L6" t="s">
-        <v>44</v>
-      </c>
-      <c r="M6">
+      <c r="M6" t="s">
+        <v>45</v>
+      </c>
+      <c r="N6">
         <v>0</v>
       </c>
-      <c r="N6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
+      <c r="O6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7" s="3">
         <v>46225</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F7">
-        <v>9.9</v>
+        <v>9.903</v>
       </c>
       <c r="G7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H7">
+        <v>1.401</v>
+      </c>
+      <c r="I7" s="1">
         <v>1.51</v>
       </c>
-      <c r="I7" s="1">
-        <v>14.95</v>
-      </c>
       <c r="J7">
+        <v>14.95353</v>
+      </c>
+      <c r="K7" s="1">
         <v>1.54</v>
       </c>
-      <c r="K7" s="1">
-        <v>15.25</v>
-      </c>
-      <c r="L7" t="s">
-        <v>45</v>
-      </c>
-      <c r="M7">
+      <c r="L7" s="1">
+        <v>15.25062</v>
+      </c>
+      <c r="M7" t="s">
+        <v>46</v>
+      </c>
+      <c r="N7">
         <v>0</v>
       </c>
-      <c r="N7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
+      <c r="O7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" s="3">
         <v>46226</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F8">
-        <v>48.05</v>
+        <v>48.052</v>
       </c>
       <c r="G8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H8">
+        <v>1.401</v>
+      </c>
+      <c r="I8" s="1">
         <v>1.51</v>
       </c>
-      <c r="I8" s="1">
-        <v>72.56</v>
-      </c>
       <c r="J8">
+        <v>72.55852</v>
+      </c>
+      <c r="K8" s="1">
         <v>1.54</v>
       </c>
-      <c r="K8" s="1">
-        <v>74</v>
-      </c>
-      <c r="L8" t="s">
-        <v>46</v>
-      </c>
-      <c r="M8">
+      <c r="L8" s="1">
+        <v>74.00008</v>
+      </c>
+      <c r="M8" t="s">
+        <v>47</v>
+      </c>
+      <c r="N8">
         <v>174237</v>
       </c>
-      <c r="N8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14">
+      <c r="O8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" s="3">
         <v>46231</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F9">
-        <v>30.85</v>
+        <v>30.851</v>
       </c>
       <c r="G9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H9">
+        <v>1.653</v>
+      </c>
+      <c r="I9" s="1">
         <v>1.72</v>
       </c>
-      <c r="I9" s="1">
-        <v>53.06</v>
-      </c>
       <c r="J9">
+        <v>53.06372</v>
+      </c>
+      <c r="K9" s="1">
         <v>1.75</v>
       </c>
-      <c r="K9" s="1">
-        <v>53.99</v>
-      </c>
-      <c r="L9" t="s">
-        <v>47</v>
-      </c>
-      <c r="M9">
+      <c r="L9" s="1">
+        <v>53.98925</v>
+      </c>
+      <c r="M9" t="s">
+        <v>48</v>
+      </c>
+      <c r="N9">
         <v>82393</v>
       </c>
-      <c r="N9" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
+      <c r="O9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" s="3">
         <v>46234</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F10">
-        <v>41.58</v>
+        <v>41.582</v>
       </c>
       <c r="G10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H10">
+        <v>1.689</v>
+      </c>
+      <c r="I10" s="1">
         <v>1.74</v>
       </c>
-      <c r="I10" s="1">
-        <v>72.34999999999999</v>
-      </c>
       <c r="J10">
+        <v>72.35268000000001</v>
+      </c>
+      <c r="K10" s="1">
         <v>1.77</v>
       </c>
-      <c r="K10" s="1">
-        <v>73.59999999999999</v>
-      </c>
-      <c r="L10" t="s">
-        <v>48</v>
-      </c>
-      <c r="M10">
+      <c r="L10" s="1">
+        <v>73.60014</v>
+      </c>
+      <c r="M10" t="s">
+        <v>49</v>
+      </c>
+      <c r="N10">
         <v>0</v>
       </c>
-      <c r="N10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
+      <c r="O10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" s="3">
         <v>46234</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F11">
-        <v>51.4</v>
+        <v>51.401</v>
       </c>
       <c r="G11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H11">
+        <v>1.689</v>
+      </c>
+      <c r="I11" s="1">
         <v>1.74</v>
       </c>
-      <c r="I11" s="1">
-        <v>89.44</v>
-      </c>
       <c r="J11">
+        <v>89.43774000000001</v>
+      </c>
+      <c r="K11" s="1">
         <v>1.77</v>
       </c>
-      <c r="K11" s="1">
-        <v>90.98</v>
-      </c>
-      <c r="L11" t="s">
-        <v>49</v>
-      </c>
-      <c r="M11">
+      <c r="L11" s="1">
+        <v>90.97977</v>
+      </c>
+      <c r="M11" t="s">
+        <v>50</v>
+      </c>
+      <c r="N11">
         <v>0</v>
       </c>
-      <c r="N11" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
+      <c r="O11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12" s="3">
         <v>46234</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F12">
-        <v>2.96</v>
+        <v>2.961</v>
       </c>
       <c r="G12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H12">
+        <v>1.459</v>
+      </c>
+      <c r="I12" s="1">
         <v>1.52</v>
       </c>
-      <c r="I12" s="1">
-        <v>4.5</v>
-      </c>
       <c r="J12">
+        <v>4.50072</v>
+      </c>
+      <c r="K12" s="1">
         <v>1.55</v>
       </c>
-      <c r="K12" s="1">
-        <v>4.59</v>
-      </c>
-      <c r="L12" t="s">
-        <v>50</v>
-      </c>
-      <c r="M12">
+      <c r="L12" s="1">
+        <v>4.58955</v>
+      </c>
+      <c r="M12" t="s">
+        <v>51</v>
+      </c>
+      <c r="N12">
         <v>49997</v>
       </c>
-      <c r="N12" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
+      <c r="O12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" s="3">
         <v>46234</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F13">
-        <v>10.16</v>
+        <v>10.158</v>
       </c>
       <c r="G13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H13">
+        <v>1.689</v>
+      </c>
+      <c r="I13" s="1">
         <v>1.74</v>
       </c>
-      <c r="I13" s="1">
-        <v>17.68</v>
-      </c>
       <c r="J13">
+        <v>17.67492</v>
+      </c>
+      <c r="K13" s="1">
         <v>1.77</v>
       </c>
-      <c r="K13" s="1">
-        <v>17.98</v>
-      </c>
-      <c r="L13" t="s">
-        <v>51</v>
-      </c>
-      <c r="M13">
+      <c r="L13" s="1">
+        <v>17.97966</v>
+      </c>
+      <c r="M13" t="s">
+        <v>52</v>
+      </c>
+      <c r="N13">
         <v>82510</v>
       </c>
-      <c r="N13" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
+      <c r="O13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" s="3">
         <v>46234</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F14">
-        <v>7.38</v>
+        <v>7.381</v>
       </c>
       <c r="G14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H14">
+        <v>1.459</v>
+      </c>
+      <c r="I14" s="1">
         <v>1.52</v>
       </c>
-      <c r="I14" s="1">
-        <v>11.22</v>
-      </c>
       <c r="J14">
+        <v>11.21912</v>
+      </c>
+      <c r="K14" s="1">
         <v>1.55</v>
       </c>
-      <c r="K14" s="1">
-        <v>11.44</v>
-      </c>
-      <c r="L14" t="s">
-        <v>52</v>
-      </c>
-      <c r="M14">
+      <c r="L14" s="1">
+        <v>11.44055</v>
+      </c>
+      <c r="M14" t="s">
+        <v>53</v>
+      </c>
+      <c r="N14">
         <v>0</v>
       </c>
-      <c r="N14" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14">
+      <c r="O14" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15" s="3">
         <v>46234</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F15">
-        <v>3.72</v>
+        <v>3.719</v>
       </c>
       <c r="G15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15" s="1">
         <v>0.63</v>
       </c>
-      <c r="I15" s="1">
-        <v>2.34</v>
-      </c>
       <c r="J15">
+        <v>2.34297</v>
+      </c>
+      <c r="K15" s="1">
         <v>0.64</v>
       </c>
-      <c r="K15" s="1">
-        <v>2.38</v>
-      </c>
-      <c r="L15" t="s">
-        <v>53</v>
-      </c>
-      <c r="M15">
+      <c r="L15" s="1">
+        <v>2.38016</v>
+      </c>
+      <c r="M15" t="s">
+        <v>54</v>
+      </c>
+      <c r="N15">
         <v>49997</v>
       </c>
-      <c r="N15" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
+      <c r="O15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16" s="3">
         <v>46234</v>
       </c>
       <c r="B16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F16">
-        <v>10.17</v>
+        <v>10.169</v>
       </c>
       <c r="G16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H16">
+        <v>1.689</v>
+      </c>
+      <c r="I16" s="1">
         <v>1.74</v>
       </c>
-      <c r="I16" s="1">
-        <v>17.7</v>
-      </c>
       <c r="J16">
+        <v>17.69406</v>
+      </c>
+      <c r="K16" s="1">
         <v>1.77</v>
       </c>
-      <c r="K16" s="1">
-        <v>18</v>
-      </c>
-      <c r="L16" t="s">
-        <v>54</v>
-      </c>
-      <c r="M16">
+      <c r="L16" s="1">
+        <v>17.99913</v>
+      </c>
+      <c r="M16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N16">
         <v>0</v>
       </c>
-      <c r="N16" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14">
+      <c r="O16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15">
       <c r="A17" s="3">
         <v>46234</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F17">
-        <v>47.06</v>
+        <v>47.062</v>
       </c>
       <c r="G17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H17">
+        <v>1.689</v>
+      </c>
+      <c r="I17" s="1">
         <v>1.74</v>
       </c>
-      <c r="I17" s="1">
-        <v>81.88</v>
-      </c>
       <c r="J17">
+        <v>81.88788</v>
+      </c>
+      <c r="K17" s="1">
         <v>1.77</v>
       </c>
-      <c r="K17" s="1">
-        <v>83.3</v>
-      </c>
-      <c r="L17" t="s">
-        <v>55</v>
-      </c>
-      <c r="M17">
+      <c r="L17" s="1">
+        <v>83.29974</v>
+      </c>
+      <c r="M17" t="s">
+        <v>56</v>
+      </c>
+      <c r="N17">
         <v>87966</v>
       </c>
-      <c r="N17" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14">
+      <c r="O17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15">
       <c r="A20" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1426,38 +1480,38 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:15">
       <c r="A21" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15">
       <c r="A22" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B22" s="7">
-        <v>299.22</v>
+        <v>299.223</v>
       </c>
       <c r="C22" s="7">
         <v>9</v>
       </c>
       <c r="D22" s="8">
-        <v>1.700555</v>
+        <v>1.700541</v>
       </c>
       <c r="E22" s="7">
         <v>508.84</v>
@@ -1466,38 +1520,38 @@
         <v>517.8200000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:15">
       <c r="A23" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B23" s="7">
-        <v>72.12</v>
+        <v>72.127</v>
       </c>
       <c r="C23" s="7">
         <v>5</v>
       </c>
       <c r="D23" s="8">
-        <v>1.510954</v>
+        <v>1.510903</v>
       </c>
       <c r="E23" s="7">
-        <v>108.97</v>
+        <v>108.98</v>
       </c>
       <c r="F23" s="7">
         <v>111.14</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:15">
       <c r="A24" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B24" s="7">
-        <v>32.78</v>
+        <v>32.782</v>
       </c>
       <c r="C24" s="7">
         <v>2</v>
       </c>
       <c r="D24" s="8">
-        <v>0.629957</v>
+        <v>0.63</v>
       </c>
       <c r="E24" s="7">
         <v>20.65</v>
@@ -1506,19 +1560,19 @@
         <v>20.98</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:15">
       <c r="A25" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B25" s="10">
-        <v>404.12</v>
+        <v>404.132</v>
       </c>
       <c r="C25" s="10">
         <v>16</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="10">
-        <v>638.46</v>
+        <v>638.47</v>
       </c>
       <c r="F25" s="10">
         <v>649.9400000000001</v>

</xml_diff>